<commit_message>
copy: call the human team the WhatsApp estate agent, not the concierge
Replaces 'concierge' with 'WhatsApp estate agent' in every WhatsApp
message, website, email, prompt, doc and data room page, and renames
the internal flags to match (needsEstateAgent, escalate_to_estate_agent,
health feature key estateAgent). The message volume model's inputs and
journey rows are renamed and the workbook rebuilt.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KVrBNQvv3TQbXwSXDnm9K8
</commit_message>
<xml_diff>
--- a/docs/whatsapp-message-volume-model.xlsx
+++ b/docs/whatsapp-message-volume-model.xlsx
@@ -45,9 +45,9 @@
     <definedName name="deals_otp">Inputs!$B$38</definedName>
     <definedName name="deals_registered">Inputs!$B$39</definedName>
     <definedName name="deadline_reminders">Inputs!$B$40</definedName>
-    <definedName name="concierge_estimate">Inputs!$B$41</definedName>
-    <definedName name="concierge_seller">Inputs!$B$42</definedName>
-    <definedName name="concierge_buyer">Inputs!$B$43</definedName>
+    <definedName name="estate_agent_estimate">Inputs!$B$41</definedName>
+    <definedName name="estate_agent_seller">Inputs!$B$42</definedName>
+    <definedName name="estate_agent_buyer">Inputs!$B$43</definedName>
     <definedName name="overhead">Inputs!$B$44</definedName>
     <definedName name="months">Inputs!$B$45</definedName>
     <definedName name="deals_Y1">Inputs!$B$48</definedName>
@@ -646,7 +646,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Charged since 1 Oct 2026 after the free tier below. Covers every scripted-flow reply and every concierge reply.</t>
+          <t>Charged since 1 Oct 2026 after the free tier below. Covers every scripted-flow reply and every WhatsApp estate agent reply.</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Concierge free-text replies per estimate contact</t>
+          <t>WhatsApp estate agent free-text replies per estimate contact</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
@@ -1227,7 +1227,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Concierge free-text replies per listed seller (over the listing's life)</t>
+          <t>WhatsApp estate agent free-text replies per listed seller (over the listing's life)</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
@@ -1247,7 +1247,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Concierge free-text replies per enquiring buyer</t>
+          <t>WhatsApp estate agent free-text replies per enquiring buyer</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
@@ -2087,7 +2087,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Concierge replies — estimate contacts</t>
+          <t>WhatsApp estate agent replies — estimate contacts</t>
         </is>
       </c>
       <c r="B16" s="8">
@@ -2095,7 +2095,7 @@
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>concierge_estimate</f>
+        <f>estate_agent_estimate</f>
         <v/>
       </c>
       <c r="D16" s="9" t="n">
@@ -2108,7 +2108,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="9">
-        <f>concierge_estimate</f>
+        <f>estate_agent_estimate</f>
         <v/>
       </c>
       <c r="H16" s="10">
@@ -2140,7 +2140,7 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Concierge replies — listed sellers</t>
+          <t>WhatsApp estate agent replies — listed sellers</t>
         </is>
       </c>
       <c r="B17" s="8">
@@ -2148,7 +2148,7 @@
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>concierge_seller</f>
+        <f>estate_agent_seller</f>
         <v/>
       </c>
       <c r="D17" s="9" t="n">
@@ -2161,7 +2161,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="9">
-        <f>concierge_seller</f>
+        <f>estate_agent_seller</f>
         <v/>
       </c>
       <c r="H17" s="10">
@@ -2189,7 +2189,7 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Concierge replies — enquiring buyers</t>
+          <t>WhatsApp estate agent replies — enquiring buyers</t>
         </is>
       </c>
       <c r="B18" s="8">
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>concierge_buyer</f>
+        <f>estate_agent_buyer</f>
         <v/>
       </c>
       <c r="D18" s="9" t="n">
@@ -2210,7 +2210,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="9">
-        <f>concierge_buyer</f>
+        <f>estate_agent_buyer</f>
         <v/>
       </c>
       <c r="H18" s="10">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>LOOM report cost (R7.50 each), Property24 subscription (R7,153/month ex VAT at the launch profile), AI concierge inference, e-signature envelopes, SMS fallback, Meta ads spend.</t>
+          <t>LOOM report cost (R7.50 each), Property24 subscription (R7,153/month ex VAT at the launch profile), AI WhatsApp estate agent inference, e-signature envelopes, SMS fallback, Meta ads spend.</t>
         </is>
       </c>
     </row>

</xml_diff>